<commit_message>
hod and exam controller
</commit_message>
<xml_diff>
--- a/sample_students.xlsx
+++ b/sample_students.xlsx
@@ -417,12 +417,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,21 +446,155 @@
           <t>password</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>program</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>semester</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>academic_year</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026001</t>
+          <t>CSE26001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sample Student</t>
+          <t>Aarav Sharma</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Exam@123</t>
+          <t>Exam@26001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>B.Tech CSE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CSE26002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ananya Verma</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Exam@26002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B.Tech CSE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CSE26003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Rohan Mehta</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Exam@26003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>B.Tech CSE</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
         </is>
       </c>
     </row>

</xml_diff>